<commit_message>
Initial commit - ExcelProject
</commit_message>
<xml_diff>
--- a/wwwroot/uploads/students.xlsx
+++ b/wwwroot/uploads/students.xlsx
@@ -47,30 +47,6 @@
   </x:si>
   <x:si>
     <x:t>Active</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mohit Modi</x:t>
-  </x:si>
-  <x:si>
-    <x:t>mohit@mail.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9427026999</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Barot Vishesh</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Vishesh@gmail.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ECE</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve"> 91577 90402</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -441,14 +417,14 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F4"/>
+  <x:dimension ref="A1:F2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="2.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13.282054" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="19.139196" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.567768" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16.282054" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.710625" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12.424911" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -489,46 +465,6 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:6">
-      <x:c r="A3" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:6">
-      <x:c r="A4" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat: lightning borders + mobile fix
</commit_message>
<xml_diff>
--- a/wwwroot/uploads/students.xlsx
+++ b/wwwroot/uploads/students.xlsx
@@ -59,6 +59,36 @@
   </x:si>
   <x:si>
     <x:t>Inactive</x:t>
+  </x:si>
+  <x:si>
+    <x:t>kirtan</x:t>
+  </x:si>
+  <x:si>
+    <x:t>kirtan@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Computer Engineering</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9427026222</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hetu</x:t>
+  </x:si>
+  <x:si>
+    <x:t>hetuhetu360@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8200640585</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jiya</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jiya@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8989898989</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -429,13 +459,13 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F3"/>
+  <x:dimension ref="A1:F6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="2.710625" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="11.567768" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16.567768" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.853482" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20.996339" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="11.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="7.996339" style="0" customWidth="1"/>
   </x:cols>
@@ -498,6 +528,66 @@
       </x:c>
       <x:c r="F3" s="0" t="s">
         <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:6">
+      <x:c r="A5" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>10</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>